<commit_message>
Refactored the excel template
</commit_message>
<xml_diff>
--- a/src/main/resources/ExcelTemplates/Sales_Quotation_Projects_Charge_Details_Template.xlsx
+++ b/src/main/resources/ExcelTemplates/Sales_Quotation_Projects_Charge_Details_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29728"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29926"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hexalytics-my.sharepoint.com/personal/hvijayakumar_hexalytics_com/Documents/Alsharif/Port Call operation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{88E268A3-D78A-4E36-B197-57169D354BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC24719A-9317-434C-8C84-523B9B110B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{3E75068D-288F-4158-AFB4-04999EE34514}"/>
   </bookViews>
@@ -41,10 +41,10 @@
     <t>SN.</t>
   </si>
   <si>
-    <t>Charge Details</t>
-  </si>
-  <si>
-    <t>Printable Charge Description</t>
+    <t>Charge Code</t>
+  </si>
+  <si>
+    <t>Charge Description</t>
   </si>
   <si>
     <t>QTY</t>
@@ -146,8 +146,8 @@
   <autoFilter ref="A2:Q3" xr:uid="{F4021E12-9FDF-4D91-B171-5CCFD12356BB}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{020D9D3F-6C47-4B26-A261-20ED23CF9486}" name="SN."/>
-    <tableColumn id="2" xr3:uid="{71B28528-6D40-4867-A145-30621204AB3F}" name="Charge Details"/>
-    <tableColumn id="3" xr3:uid="{55F83E29-4879-4A9F-8DB0-16F7F36ACA3D}" name="Printable Charge Description"/>
+    <tableColumn id="2" xr3:uid="{71B28528-6D40-4867-A145-30621204AB3F}" name="Charge Code"/>
+    <tableColumn id="3" xr3:uid="{55F83E29-4879-4A9F-8DB0-16F7F36ACA3D}" name="Charge Description"/>
     <tableColumn id="4" xr3:uid="{9D9AAE44-2052-4527-AB3B-437AEC193C94}" name="QTY"/>
     <tableColumn id="5" xr3:uid="{A893A968-7A6F-4E89-BE57-401337CA87C1}" name="Unit"/>
     <tableColumn id="16" xr3:uid="{F1CD15E3-6986-43A8-8B86-0931F2890939}" name="Buying Currency"/>

</xml_diff>